<commit_message>
Last graphs for comparaison rest of the economy
</commit_message>
<xml_diff>
--- a/data/data_minerals/data_availability_marin.xlsx
+++ b/data/data_minerals/data_availability_marin.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polymtlca0-my.sharepoint.com/personal/marin_pellan_polymtlus_ca/Documents/Desktop/POST_DOC/Project/plca_metals_github/plca_metals/data/data_minerals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2440" documentId="13_ncr:1_{3B0093C0-0E66-4485-936E-AE5475C25BEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AFE3B620-6845-46C1-B4CD-9FCABA397A71}"/>
+  <xr:revisionPtr revIDLastSave="2442" documentId="13_ncr:1_{3B0093C0-0E66-4485-936E-AE5475C25BEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9ED8C0DA-D407-4C1E-8056-4989AA6362BE}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="7" r:id="rId1"/>
@@ -4054,15 +4054,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:colOff>18203</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>34853</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>213956</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>38527</xdr:rowOff>
+      <xdr:colOff>192789</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>30200</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4085,8 +4085,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3345180" y="3703320"/>
-          <a:ext cx="6881456" cy="4930567"/>
+          <a:off x="3313147" y="4804409"/>
+          <a:ext cx="6849142" cy="4948347"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4096,6 +4096,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>